<commit_message>
feat: Add a glossary section to generated keyword reports and introduce a new script to merge multiple reports into a single Excel file.
</commit_message>
<xml_diff>
--- a/destination/Cát Bà - keyword.xlsx
+++ b/destination/Cát Bà - keyword.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -45,6 +45,11 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -106,7 +111,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -127,6 +132,8 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -492,7 +499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I116"/>
+  <dimension ref="A1:I137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5347,19 +5354,163 @@
         </is>
       </c>
     </row>
+    <row r="119">
+      <c r="A119" s="2" t="inlineStr">
+        <is>
+          <t>4. CHÚ THÍCH GIẢI NGHĨA CÁC CỘT</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="8" t="inlineStr">
+        <is>
+          <t>--- Nhóm A ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="9" t="inlineStr">
+        <is>
+          <t>- Cluster: Nhóm chủ đề</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="9" t="inlineStr">
+        <is>
+          <t>- Cluster type: Nhóm từ khoá của chủ đề</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="9" t="inlineStr">
+        <is>
+          <t>- Keyword: Từ khoá để SEO</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="9" t="inlineStr">
+        <is>
+          <t>- Intent: Mục đích, ý định tìm kiếm của khách hàng</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="9" t="inlineStr">
+        <is>
+          <t>- Impression: Số lần Vietgoing hiển thị cho 1 từ khoá cụ thể (Thông thường là ở page 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="9" t="inlineStr">
+        <is>
+          <t>- Clicks: Số lượt truy cập vào website Vietgoing cho 1 từ khoá cụ thể</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="9" t="inlineStr">
+        <is>
+          <t>- Source: Nguồn dữ liệu</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="8" t="inlineStr">
+        <is>
+          <t>--- Nhóm B ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="9" t="inlineStr">
+        <is>
+          <t>- Cluster: Nhóm chủ đề</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="9" t="inlineStr">
+        <is>
+          <t>- Cluster type: Nhóm từ khoá của chủ đề</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="9" t="inlineStr">
+        <is>
+          <t>- Keyword: Từ khoá để SEO</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="9" t="inlineStr">
+        <is>
+          <t>- Intent: Mục đích, ý định tìm kiếm của khách hàng</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="9" t="inlineStr">
+        <is>
+          <t>- Vol: Lưu lượng tìm kiếm của từ khoá</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="9" t="inlineStr">
+        <is>
+          <t>- YoY: Tăng trưởng tìm kiếm của từ khoá</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="9" t="inlineStr">
+        <is>
+          <t>- KD/Comp: Tính cạnh tranh cho từ khoá</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="9" t="inlineStr">
+        <is>
+          <t>- Bid: Giá thầu dự kiến trên Google Ads (High)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="29">
     <mergeCell ref="A7:I7"/>
-    <mergeCell ref="A10:I10"/>
+    <mergeCell ref="A137:I137"/>
+    <mergeCell ref="A133:I133"/>
+    <mergeCell ref="A120:I120"/>
+    <mergeCell ref="A3:I3"/>
+    <mergeCell ref="A136:I136"/>
+    <mergeCell ref="A12:I12"/>
+    <mergeCell ref="A129:I129"/>
     <mergeCell ref="A5:I5"/>
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A9:I9"/>
+    <mergeCell ref="A126:I126"/>
     <mergeCell ref="A8:I8"/>
-    <mergeCell ref="A3:I3"/>
-    <mergeCell ref="A6:I6"/>
-    <mergeCell ref="A12:I12"/>
+    <mergeCell ref="A122:I122"/>
+    <mergeCell ref="A135:I135"/>
+    <mergeCell ref="A131:I131"/>
     <mergeCell ref="A4:I4"/>
     <mergeCell ref="A20:I20"/>
+    <mergeCell ref="A125:I125"/>
+    <mergeCell ref="A134:I134"/>
+    <mergeCell ref="A121:I121"/>
+    <mergeCell ref="A10:I10"/>
+    <mergeCell ref="A127:I127"/>
+    <mergeCell ref="A9:I9"/>
+    <mergeCell ref="A130:I130"/>
+    <mergeCell ref="A123:I123"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A132:I132"/>
+    <mergeCell ref="A124:I124"/>
+    <mergeCell ref="A6:I6"/>
+    <mergeCell ref="A119:I119"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>